<commit_message>
docs: completar Diccionario_de_datos y Preguntas con las mejoras de Milan e integracion territorial
</commit_message>
<xml_diff>
--- a/Diccionario_de_datos_TallerDatos.xlsx
+++ b/Diccionario_de_datos_TallerDatos.xlsx
@@ -567,28 +567,28 @@
     <row r="4" ht="16" customHeight="1">
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Milán (Milano, Italia)</t>
+          <t>Datos del grupo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Ciudad elegida:</t>
+          <t>Ciudad elegida: Milán (Milano, Italia)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Integrantes:</t>
+          <t>Integrantes: Alyson Henao, Mateo Sanz, Samuel Arango, Emily Cardona</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Enlace al repositorio o a la carpeta del lago:</t>
+          <t>Enlace al repositorio o a la carpeta del lago: https://github.com/MateoSanzEafit/CerebroMilan</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>CSV</t>
+          <t>CSV / GeoJSON</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="M5" s="10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N5" s="10" t="inlineStr">
@@ -963,12 +963,12 @@
       </c>
       <c r="O5" s="10" t="inlineStr">
         <is>
-          <t>Búsqueda en catálogo oficial CKAN (name:nil)</t>
+          <t>Búsqueda en catálogo oficial CKAN del Comune (name:nil)</t>
         </is>
       </c>
       <c r="P5" s="10" t="inlineStr">
         <is>
-          <t>Malla territorial oficial de los 88 barrios/núcleos con centroides WGS84 (EPSG:4326). Base geométrica del gemelo.</t>
+          <t>Malla territorial oficial aprobada por el PGT 2030 con geometrías vectoriales y centroides WGS84 (EPSG:4326).</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>CSV</t>
+          <t>CSV (ZIP) / JSON</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>Creative Commons Attribution</t>
+          <t>Creative Commons Attribution (CC-BY 4.0)</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="M6" s="10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N6" s="10" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t>Serie histórica de residentes y familias por barrio. Responde a la pregunta de densidad demográfica y presión residencial.</t>
+          <t>Serie histórica oficial de hogares y familias censadas sin microdatos personales.</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>CSV</t>
+          <t>CSV / JSON</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>Creative Commons Attribution</t>
+          <t>Creative Commons Attribution (CC-BY 4.0)</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="M7" s="10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N7" s="10" t="inlineStr">
@@ -1127,12 +1127,12 @@
       </c>
       <c r="O7" s="10" t="inlineStr">
         <is>
-          <t>Búsqueda CKAN (incidenti stradali)</t>
+          <t>Búsqueda en catálogo CKAN (incidenti stradali)</t>
         </is>
       </c>
       <c r="P7" s="10" t="inlineStr">
         <is>
-          <t>Siniestros viales clasificados en incidentes, heridos y fallecidos por mes y municipio de descentramiento.</t>
+          <t>Conteo mensual de siniestros, personas lesionadas y víctimas fatales agregado por municipio para evitar reidentificación.</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="M8" s="10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N8" s="10" t="inlineStr">
@@ -1209,12 +1209,12 @@
       </c>
       <c r="O8" s="10" t="inlineStr">
         <is>
-          <t>Búsqueda CKAN (bikemi)</t>
+          <t>Búsqueda CKAN oficial (bikemi)</t>
         </is>
       </c>
       <c r="P8" s="10" t="inlineStr">
         <is>
-          <t>Estaciones georreferenciadas con número de anclajes de bicis mecánicas y eléctricas para movilidad activa.</t>
+          <t>325 estaciones georreferenciadas con número de anclajes de bicis tradicionales y eléctricas para movilidad activa.</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="M9" s="10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N9" s="10" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="P9" s="10" t="inlineStr">
         <is>
-          <t>Trazados vectoriales de carriles y pistas ciclistas. Permite contrastar oferta de movilidad limpia vs. accidentes viales.</t>
+          <t>Trazados vectoriales de la red ciclista protegida y compartida para contrastar infraestructura vs accidentes.</t>
         </is>
       </c>
     </row>
@@ -1323,12 +1323,12 @@
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>https://dati.comune.milano.it/dataset/884b70a5-951c-4c92-931e-52a73d20af9f/resource/1af3c7d2-3456-4f7c-819a-464c989b9ed5/download/qaria_datoariagiornostazione_2026-09-26.csv</t>
+          <t>https://dati.comune.milano.it/dataset/884b70a5-951c-4c92-931e-52a73d20af9f/resource/ddecb297-6e09-456e-aed3-7c934eec4dd3/download/qaria_datoariagiornostazione_2026-09-26.json</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>CSV</t>
+          <t>JSON</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>Creative Commons Attribution</t>
+          <t>Creative Commons Attribution (CC-BY 4.0)</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="M10" s="10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N10" s="10" t="inlineStr">
@@ -1373,12 +1373,12 @@
       </c>
       <c r="O10" s="10" t="inlineStr">
         <is>
-          <t>Búsqueda CKAN (qualita aria 2026)</t>
+          <t>Búsqueda CKAN oficial tras descartar endpoint ficticio de IA (ds2969)</t>
         </is>
       </c>
       <c r="P10" s="10" t="inlineStr">
         <is>
-          <t>Monitoreo ambiental al día: niveles diarios de NO2, PM10, PM2.5 y C6H6 en estaciones urbanas.</t>
+          <t>Monitoreo diario oficial de contaminantes críticos urbanos (NO2, PM10, PM2.5, C6H6).</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1445,7 @@
       </c>
       <c r="M11" s="10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N11" s="10" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="P11" s="10" t="inlineStr">
         <is>
-          <t>Cámaras de acceso y control ambiental a la mayor zona de tráfico restringido de Italia.</t>
+          <t>188 cámaras de control perimetral vehicular utilizadas como proxy de presión de tráfico y emisiones.</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>Creative Commons Attribution</t>
+          <t>Creative Commons Attribution (CC-BY 4.0)</t>
         </is>
       </c>
       <c r="I12" s="10" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="M12" s="10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N12" s="10" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="P12" s="10" t="inlineStr">
         <is>
-          <t>Histórico de alojamientos y camas por categoría. Sirve para evaluar presión turística sobre vivienda.</t>
+          <t>Histórico de alojamientos y camas por categoría para evaluar presión turística sobre vivienda.</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="M13" s="10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N13" s="10" t="inlineStr">
@@ -1619,12 +1619,12 @@
       </c>
       <c r="O13" s="10" t="inlineStr">
         <is>
-          <t>Script de consulta curl / requests</t>
+          <t>Script de consulta REST verificado con curl y URL canónica codificada</t>
         </is>
       </c>
       <c r="P13" s="10" t="inlineStr">
         <is>
-          <t>Métrica de escucha social: interés global en la ciudad, filtrando tráfico no humano (user).</t>
+          <t>Métrica de escucha social: interés global en Milán excluyendo bots y crawlers (filtro agent: user).</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="M14" s="10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N14" s="10" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="P14" s="10" t="inlineStr">
         <is>
-          <t>DESCARTADA: expone nombres de directivos, correos electrónicos directos y teléfonos. Se descarta por minimización y privacidad (RGPD / Ley 1581).</t>
+          <t>DESCARTADA: expone nombres de directivos, correos (@psicologoalparco.it) y celulares directos. Violación de minimización y RGPD / Ley 1581.</t>
         </is>
       </c>
     </row>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="M15" s="10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N15" s="10" t="inlineStr">
@@ -2547,10 +2547,8 @@
           <t>visitas de usuarios</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>13195</t>
-        </is>
+      <c r="H5" s="10" t="n">
+        <v>13195</v>
       </c>
       <c r="I5" s="10" t="inlineStr">
         <is>
@@ -2559,7 +2557,7 @@
       </c>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>&gt;= 0</t>
+          <t>≥ 0</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
@@ -2614,10 +2612,8 @@
           <t>siniestros viales</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>7602</t>
-        </is>
+      <c r="H6" s="10" t="n">
+        <v>7602</v>
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
@@ -2626,7 +2622,7 @@
       </c>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>&gt;= 0</t>
+          <t>≥ 0</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
@@ -2681,10 +2677,8 @@
           <t>personas lesionadas</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>9384</t>
-        </is>
+      <c r="H7" s="10" t="n">
+        <v>9384</v>
       </c>
       <c r="I7" s="10" t="inlineStr">
         <is>
@@ -2693,7 +2687,7 @@
       </c>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>&gt;= 0</t>
+          <t>≥ 0</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
@@ -2748,10 +2742,8 @@
           <t>familias censadas</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>620587</t>
-        </is>
+      <c r="H8" s="10" t="n">
+        <v>620587</v>
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
@@ -2760,7 +2752,7 @@
       </c>
       <c r="J8" s="10" t="inlineStr">
         <is>
-          <t>&gt;= 0</t>
+          <t>≥ 0</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
@@ -2815,10 +2807,8 @@
           <t>habitantes en familias</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>1002644</t>
-        </is>
+      <c r="H9" s="10" t="n">
+        <v>1002644</v>
       </c>
       <c r="I9" s="10" t="inlineStr">
         <is>
@@ -2827,7 +2817,7 @@
       </c>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>&gt;= 0</t>
+          <t>≥ 0</t>
         </is>
       </c>
       <c r="K9" s="10" t="inlineStr">
@@ -2882,10 +2872,8 @@
           <t>µg/m³</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>59.92</t>
-        </is>
+      <c r="H10" s="10" t="n">
+        <v>59.92</v>
       </c>
       <c r="I10" s="10" t="inlineStr">
         <is>
@@ -2894,7 +2882,7 @@
       </c>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t>&gt;= 0.0</t>
+          <t>≥ 0.0</t>
         </is>
       </c>
       <c r="K10" s="10" t="inlineStr">
@@ -2949,10 +2937,8 @@
           <t>µg/m³</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>30.40</t>
-        </is>
+      <c r="H11" s="10" t="n">
+        <v>30.4</v>
       </c>
       <c r="I11" s="10" t="inlineStr">
         <is>
@@ -2961,7 +2947,7 @@
       </c>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>&gt;= 0.0</t>
+          <t>≥ 0.0</t>
         </is>
       </c>
       <c r="K11" s="10" t="inlineStr">
@@ -3016,10 +3002,8 @@
           <t>código territorial</t>
         </is>
       </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
+      <c r="H12" s="10" t="n">
+        <v>48</v>
       </c>
       <c r="I12" s="10" t="inlineStr">
         <is>
@@ -3048,64 +3032,268 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
-      <c r="H13" s="10" t="n"/>
-      <c r="I13" s="10" t="n"/>
-      <c r="J13" s="10" t="n"/>
-      <c r="K13" s="10" t="n"/>
-      <c r="L13" s="10" t="n"/>
-      <c r="M13" s="10" t="n"/>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>territorio/nil.geojson</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>nombre_nil</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>NIL</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Denominación toponímica oficial del barrio según el Plan General de Territorio (PGT 2030)</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>nombre de barrio</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>DUOMO</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>Texto oficial PGT</t>
+        </is>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>Pública</t>
+        </is>
+      </c>
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>Normalización en mayúsculas sostenidas y codificación UTF-8</t>
+        </is>
+      </c>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t>¿Cómo se denomina y delimita cada uno de los 88 barrios de Milán?</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
-      <c r="H14" s="10" t="n"/>
-      <c r="I14" s="10" t="n"/>
-      <c r="J14" s="10" t="n"/>
-      <c r="K14" s="10" t="n"/>
-      <c r="L14" s="10" t="n"/>
-      <c r="M14" s="10" t="n"/>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>territorio/nil.geojson</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>superficie_nil_m2</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Shape_Area</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Área territorial total en metros cuadrados del polígono barrial en proyección oficial</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>Decimal</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>metros cuadrados (m²)</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>2406306.08</v>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J14" s="10" t="inlineStr">
+        <is>
+          <t>&gt; 0.0</t>
+        </is>
+      </c>
+      <c r="K14" s="10" t="inlineStr">
+        <is>
+          <t>Pública</t>
+        </is>
+      </c>
+      <c r="L14" s="10" t="inlineStr">
+        <is>
+          <t>Cálculo geométrico del polígono proyectado en EPSG:4326</t>
+        </is>
+      </c>
+      <c r="M14" s="10" t="inlineStr">
+        <is>
+          <t>¿Cuál es la extensión espacial de cada núcleo de identidad local?</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="10" t="n"/>
-      <c r="I15" s="10" t="n"/>
-      <c r="J15" s="10" t="n"/>
-      <c r="K15" s="10" t="n"/>
-      <c r="L15" s="10" t="n"/>
-      <c r="M15" s="10" t="n"/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>territorio/bikemi.geojson</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>id_estacion_bikemi</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>numero</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Número identificador oficial de la estación de bicicletas públicas compartidas BikeMi</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>código de estación</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>102</v>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
+        <is>
+          <t>1 a 500</t>
+        </is>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
+        <is>
+          <t>Pública</t>
+        </is>
+      </c>
+      <c r="L15" s="10" t="inlineStr">
+        <is>
+          <t>Validación de código numérico entero asignado por AMAT</t>
+        </is>
+      </c>
+      <c r="M15" s="10" t="inlineStr">
+        <is>
+          <t>¿Cómo se distribuye la infraestructura de micromovilidad en la ciudad?</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
-      <c r="H16" s="10" t="n"/>
-      <c r="I16" s="10" t="n"/>
-      <c r="J16" s="10" t="n"/>
-      <c r="K16" s="10" t="n"/>
-      <c r="L16" s="10" t="n"/>
-      <c r="M16" s="10" t="n"/>
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>territorio/bikemi.geojson</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>nombre_estacion</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Dirección y referencia física de localización del punto de anclaje de bicicletas</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>dirección toponímica</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>Cordusio</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>Texto no vacío</t>
+        </is>
+      </c>
+      <c r="K16" s="10" t="inlineStr">
+        <is>
+          <t>Pública</t>
+        </is>
+      </c>
+      <c r="L16" s="10" t="inlineStr">
+        <is>
+          <t>Normalización de cadenas y limpieza de espacios en blanco</t>
+        </is>
+      </c>
+      <c r="M16" s="10" t="inlineStr">
+        <is>
+          <t>¿Dónde están ubicadas las estaciones de bicicletas compartidas?</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n"/>
@@ -3660,192 +3848,244 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A5" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Encontrar una fuente abierta y sin llave que mida cuánto interés despierta Milán fuera de Italia</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Propuso Google Trends y la API de vistas de Wikipedia</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Probamos las dos: Google Trends no tiene API abierta ni licencia de reutilización; la de Wikimedia respondió con curl y declara CC0</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Que la IA mencione una fuente no implica que se pueda usar: la licencia y el acceso se auditan empíricamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
           <t>Claude Code / Antigravity</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Localizar la escala y subdivisión territorial oficial de Milán para estructurar el gemelo urbano</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Sugirió buscar por 'distretti' genéricos o comunas metropolitanas</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>Consultamos la documentación del Comune y descubrimos que la unidad oficial de planificación son los 88 NIL (Nuclei di Identità Locale)</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Consultamos la documentación oficial del Comune di Milano y descubrimos que la unidad oficial de planificación son los 88 NIL (Nuclei di Identità Locale) aprobados por el PGT 2030</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>F01</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>Milán no divide su planificación en distritos como Lima; su unidad oficial normativa aprobada en el PGT son los NIL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Milán no divide su planificación territorial en distritos genéricos como Lima; su unidad oficial normativa aprobada en el PGT son los NIL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Claude Code / Antigravity</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Encontrar una API oficial en tiempo real de calidad del aire para Milán</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Inventó un endpoint inexistente: https://dati.comune.milano.it/api/v1/airquality/stations.json</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>Probamos la URL con curl y devolvió error 404; auditamos el catálogo CKAN hasta encontrar el recurso vigente ds2969 (septiembre 2026)</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Probamos la URL con curl y devolvió error HTTP 404; auditamos el catálogo CKAN oficial hasta encontrar el recurso vigente ds2969 (septiembre 2026)</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>Inventado</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="G7" s="10" t="inlineStr">
         <is>
           <t>F06</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H7" s="10" t="inlineStr">
         <is>
           <t>Los modelos de lenguaje inventan rutas REST verosímiles; ninguna URL entra al catálogo sin comprobarse en la terminal.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Claude Code / Antigravity</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Escribir el script de ingesta de consultas mensuales en Wikipedia para Milán</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Entregó código estándar con urllib pero con la URL sin codificar para caracteres especiales ('Milán')</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>La API de Wikimedia falló con desambiguación; se corrigió agregando urllib.parse.quote y resolviendo el título canónico</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>La API de Wikimedia falló con página de desambiguación; se corrigió agregando urllib.parse.quote y resolviendo el título canónico normalizado</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>F09</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>Los títulos con tildes requieren codificación de URL canónica para no romper la reproducibilidad del script.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Los títulos con tildes y caracteres especiales requieren codificación canónica de URL para garantizar reproducibilidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Claude Code / Antigravity</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Generar expresión regular para verificar ausencia de datos personales (PII) en el lago</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>Propuso un regex diseñado exclusivamente para celulares de Colombia (3\d{9})</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Propuso un regex diseñado exclusivamente para números celulares de Colombia (3\d{9})</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>Nos dimos cuenta de que dejaría pasar números italianos; lo corregimos incorporando prefijos internacionales y móviles de Italia ((?:\+39\s?)?3\d{8,9})</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G9" s="10" t="inlineStr">
         <is>
           <t>F10</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H9" s="10" t="inlineStr">
         <is>
           <t>Las políticas y filtros de seguridad como código deben ajustarse a la normativa y territorio del sistema que se gobierna.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="10" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
-      <c r="H9" s="10" t="n"/>
-    </row>
     <row r="10">
-      <c r="A10" s="10" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="10" t="n"/>
+      <c r="A10" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>ChatGPT-4o</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Rastrear telemetría de consumo eléctrico y gas en tiempo real por cada barrio (NIL) de Milán</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Afirmó que la empresa de servicios públicos A2A publicaba una API REST abierta en a2a.eu/opendata/energy-nil.json</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Se probó con curl: el dominio devolvió HTTP 404 y tras contactar el portal se constató que la telemetría energética es información comercial reservada</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Inventado</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>F07</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>La IA inventa accesos abiertos para datos que son privados o comerciales; obligó a diseñar la solución sustituta mediante proxies de Área B y NO2.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="n"/>

</xml_diff>